<commit_message>
Update Escanor, The Driller, Knuckle, Morgott, and Batman; polish My Deck
Escanor "The One": rename to Escanor.
The Driller: change origin from MCU to Transformers; retain chapter eighteen reward as filler.
APR: rename to Knuckle; retain its two-turn attack lock.
Margit the Fell Omen: replace the collectible with Morgott, the Omen King, a 3-mana 1/1 with Taunt and Battlecry: summon a 1/1 Taunt Margit. Remove the old Deathrattle and use the existing Morgott artwork.
Batman: change origin from DCU to DCEU.

Refresh the single workbook and lore. Add immediate green deck outlines and a themed cursor; remove add-card hover messages and the save reminder. Repair campaign classification and state-based verification. Check bot legality in the current thirty-card format.
</commit_message>
<xml_diff>
--- a/materials/Convergence card stat excel sheet.xlsx
+++ b/materials/Convergence card stat excel sheet.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cards" sheetId="1" r:id="R46e2905169bf4d51"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relics" sheetId="2" r:id="R78ef6e0b3061448a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rules" sheetId="3" r:id="R66541e5d5dfa41c6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="4" r:id="R406e04dc87394afc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cards" sheetId="1" r:id="R4ff3da13036949a9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relics" sheetId="2" r:id="R660a50aa63bf4fd5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rules" sheetId="3" r:id="Re7486e469968433e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="4" r:id="R49602fe1e1e84cb0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1559,7 +1559,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="B28" s="14" t="str">
-        <x:v>Escanor "The One"</x:v>
+        <x:v>Escanor</x:v>
       </x:c>
       <x:c r="C28" s="23" t="str">
         <x:f>D28&amp;"/"&amp;E28</x:f>
@@ -4278,7 +4278,7 @@
         <x:v>Latest design</x:v>
       </x:c>
       <x:c r="K97" s="18" t="str">
-        <x:v>MCU</x:v>
+        <x:v>Transformers</x:v>
       </x:c>
       <x:c r="L97" s="17" t="str">
         <x:v>c105</x:v>
@@ -5454,82 +5454,82 @@
         <x:v>c125</x:v>
       </x:c>
     </x:row>
-    <x:row r="128" ht="44" customHeight="1">
+    <x:row r="128" ht="42" customHeight="1">
       <x:c r="A128" s="21" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="B128" s="14" t="str">
-        <x:v>APR</x:v>
+        <x:v>Dabi</x:v>
       </x:c>
       <x:c r="C128" s="23" t="str">
         <x:f>D128&amp;"/"&amp;E128</x:f>
-        <x:v>0/3</x:v>
+        <x:v>3/3</x:v>
       </x:c>
       <x:c r="D128" s="21" t="n">
-        <x:v>0</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="E128" s="21" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="F128" s="23" t="str">
-        <x:v>Rare</x:v>
+        <x:v>Epic</x:v>
       </x:c>
       <x:c r="G128" s="23" t="str">
         <x:v>Magic</x:v>
       </x:c>
       <x:c r="H128" s="23" t="str">
-        <x:v>Good</x:v>
+        <x:v>Evil</x:v>
       </x:c>
       <x:c r="I128" s="13" t="str">
-        <x:v>Taunt. Passive: After the enemy minion attacks this minion, it can't attack for 2 turns</x:v>
+        <x:v>Battlecry: Deal 1 damage to all other minions</x:v>
       </x:c>
       <x:c r="J128" s="13" t="str">
-        <x:v>Taxes</x:v>
+        <x:v>He burns with anger</x:v>
       </x:c>
       <x:c r="K128" s="13" t="str">
-        <x:v>HxH</x:v>
+        <x:v>MHA</x:v>
       </x:c>
       <x:c r="L128" s="12" t="str">
-        <x:v>c135</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="129" ht="42" customHeight="1">
+        <x:v>c129</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="129" ht="44" customHeight="1">
       <x:c r="A129" s="22" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="B129" s="19" t="str">
-        <x:v>Dabi</x:v>
+        <x:v>Darkwing</x:v>
       </x:c>
       <x:c r="C129" s="24" t="str">
         <x:f>D129&amp;"/"&amp;E129</x:f>
-        <x:v>3/3</x:v>
+        <x:v>2/2</x:v>
       </x:c>
       <x:c r="D129" s="22" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="E129" s="22" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F129" s="24" t="str">
-        <x:v>Epic</x:v>
+        <x:v>Mythic</x:v>
       </x:c>
       <x:c r="G129" s="24" t="str">
-        <x:v>Magic</x:v>
+        <x:v>Tech</x:v>
       </x:c>
       <x:c r="H129" s="24" t="str">
-        <x:v>Evil</x:v>
+        <x:v>Good</x:v>
       </x:c>
       <x:c r="I129" s="18" t="str">
-        <x:v>Battlecry: Deal 1 damage to all other minions</x:v>
+        <x:v>Deathrattle: The minion which kills this minion also dies right after</x:v>
       </x:c>
       <x:c r="J129" s="18" t="str">
-        <x:v>He burns with anger</x:v>
+        <x:v>He knew the cost</x:v>
       </x:c>
       <x:c r="K129" s="18" t="str">
-        <x:v>MHA</x:v>
+        <x:v>Invincible</x:v>
       </x:c>
       <x:c r="L129" s="17" t="str">
-        <x:v>c129</x:v>
+        <x:v>c123</x:v>
       </x:c>
     </x:row>
     <x:row r="130" ht="44" customHeight="1">
@@ -5537,46 +5537,46 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B130" s="14" t="str">
-        <x:v>Darkwing</x:v>
+        <x:v>Giant Crystal</x:v>
       </x:c>
       <x:c r="C130" s="23" t="str">
         <x:f>D130&amp;"/"&amp;E130</x:f>
-        <x:v>2/2</x:v>
+        <x:v>1/1</x:v>
       </x:c>
       <x:c r="D130" s="21" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E130" s="21" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F130" s="23" t="str">
-        <x:v>Mythic</x:v>
+        <x:v>Rare</x:v>
       </x:c>
       <x:c r="G130" s="23" t="str">
-        <x:v>Tech</x:v>
+        <x:v>Magic</x:v>
       </x:c>
       <x:c r="H130" s="23" t="str">
-        <x:v>Good</x:v>
+        <x:v>Neutral</x:v>
       </x:c>
       <x:c r="I130" s="13" t="str">
-        <x:v>Deathrattle: The minion which kills this minion also dies right after</x:v>
+        <x:v>Divine Shield. Ongoing: Give all other friendly Magic minions +2/+1</x:v>
       </x:c>
       <x:c r="J130" s="13" t="str">
-        <x:v>He knew the cost</x:v>
+        <x:v>Spawnpoint</x:v>
       </x:c>
       <x:c r="K130" s="13" t="str">
-        <x:v>Invincible</x:v>
+        <x:v>Core</x:v>
       </x:c>
       <x:c r="L130" s="12" t="str">
-        <x:v>c123</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="131" ht="44" customHeight="1">
+        <x:v>c137</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="131" ht="42" customHeight="1">
       <x:c r="A131" s="22" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="B131" s="19" t="str">
-        <x:v>Giant Crystal</x:v>
+        <x:v>Giant Tree</x:v>
       </x:c>
       <x:c r="C131" s="24" t="str">
         <x:f>D131&amp;"/"&amp;E131</x:f>
@@ -5592,100 +5592,100 @@
         <x:v>Rare</x:v>
       </x:c>
       <x:c r="G131" s="24" t="str">
-        <x:v>Magic</x:v>
+        <x:v>Nature</x:v>
       </x:c>
       <x:c r="H131" s="24" t="str">
         <x:v>Neutral</x:v>
       </x:c>
       <x:c r="I131" s="18" t="str">
-        <x:v>Divine Shield. Ongoing: Give all other friendly Magic minions +2/+1</x:v>
+        <x:v>Passive: All other friendly Nature minions have +2/+1</x:v>
       </x:c>
       <x:c r="J131" s="18" t="str">
-        <x:v>Spawnpoint</x:v>
+        <x:v>Older than the roots it feeds.</x:v>
       </x:c>
       <x:c r="K131" s="18" t="str">
         <x:v>Core</x:v>
       </x:c>
       <x:c r="L131" s="17" t="str">
-        <x:v>c137</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="132" ht="42" customHeight="1">
+        <x:v>c138</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="132" ht="44" customHeight="1">
       <x:c r="A132" s="21" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="B132" s="14" t="str">
-        <x:v>Giant Tree</x:v>
+        <x:v>Godrick the Grafted</x:v>
       </x:c>
       <x:c r="C132" s="23" t="str">
         <x:f>D132&amp;"/"&amp;E132</x:f>
-        <x:v>1/1</x:v>
+        <x:v>2/2</x:v>
       </x:c>
       <x:c r="D132" s="21" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="E132" s="21" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F132" s="23" t="str">
-        <x:v>Rare</x:v>
+        <x:v>Epic</x:v>
       </x:c>
       <x:c r="G132" s="23" t="str">
-        <x:v>Nature</x:v>
+        <x:v>Magic</x:v>
       </x:c>
       <x:c r="H132" s="23" t="str">
-        <x:v>Neutral</x:v>
+        <x:v>Evil</x:v>
       </x:c>
       <x:c r="I132" s="13" t="str">
-        <x:v>Passive: All other friendly Nature minions have +2/+1</x:v>
+        <x:v>Battlecry: Destroy a friendly minion to gain its stats and effects</x:v>
       </x:c>
       <x:c r="J132" s="13" t="str">
-        <x:v>Older than the roots it feeds.</x:v>
+        <x:v>Grafted</x:v>
       </x:c>
       <x:c r="K132" s="13" t="str">
-        <x:v>Core</x:v>
+        <x:v>Elden Ring</x:v>
       </x:c>
       <x:c r="L132" s="12" t="str">
-        <x:v>c138</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="133" ht="44" customHeight="1">
+        <x:v>c130</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="133" ht="42" customHeight="1">
       <x:c r="A133" s="22" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="B133" s="19" t="str">
-        <x:v>Godrick the Grafted</x:v>
+        <x:v>Gums</x:v>
       </x:c>
       <x:c r="C133" s="24" t="str">
         <x:f>D133&amp;"/"&amp;E133</x:f>
-        <x:v>2/2</x:v>
+        <x:v>1/1</x:v>
       </x:c>
       <x:c r="D133" s="22" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E133" s="22" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F133" s="24" t="str">
-        <x:v>Epic</x:v>
+        <x:v>Legendary</x:v>
       </x:c>
       <x:c r="G133" s="24" t="str">
-        <x:v>Magic</x:v>
+        <x:v>Nature</x:v>
       </x:c>
       <x:c r="H133" s="24" t="str">
         <x:v>Evil</x:v>
       </x:c>
       <x:c r="I133" s="18" t="str">
-        <x:v>Battlecry: Destroy a friendly minion to gain its stats and effects</x:v>
+        <x:v>Battlecry: Consume an enemy Nature minion with 4 HP or lower</x:v>
       </x:c>
       <x:c r="J133" s="18" t="str">
-        <x:v>Grafted</x:v>
+        <x:v>Insatiable hunger</x:v>
       </x:c>
       <x:c r="K133" s="18" t="str">
-        <x:v>Elden Ring</x:v>
+        <x:v>OPM</x:v>
       </x:c>
       <x:c r="L133" s="17" t="str">
-        <x:v>c130</x:v>
+        <x:v>c126</x:v>
       </x:c>
     </x:row>
     <x:row r="134" ht="42" customHeight="1">
@@ -5693,7 +5693,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B134" s="14" t="str">
-        <x:v>Gums</x:v>
+        <x:v>Illumi</x:v>
       </x:c>
       <x:c r="C134" s="23" t="str">
         <x:f>D134&amp;"/"&amp;E134</x:f>
@@ -5706,25 +5706,25 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="F134" s="23" t="str">
-        <x:v>Legendary</x:v>
+        <x:v>Epic</x:v>
       </x:c>
       <x:c r="G134" s="23" t="str">
-        <x:v>Nature</x:v>
+        <x:v>Magic</x:v>
       </x:c>
       <x:c r="H134" s="23" t="str">
         <x:v>Evil</x:v>
       </x:c>
       <x:c r="I134" s="13" t="str">
-        <x:v>Battlecry: Consume an enemy Nature minion with 4 HP or lower</x:v>
+        <x:v>Battlecry: Gain control of a minion with 2 HP or less</x:v>
       </x:c>
       <x:c r="J134" s="13" t="str">
-        <x:v>Insatiable hunger</x:v>
+        <x:v>Control</x:v>
       </x:c>
       <x:c r="K134" s="13" t="str">
-        <x:v>OPM</x:v>
+        <x:v>HxH</x:v>
       </x:c>
       <x:c r="L134" s="12" t="str">
-        <x:v>c126</x:v>
+        <x:v>c131</x:v>
       </x:c>
     </x:row>
     <x:row r="135" ht="42" customHeight="1">
@@ -5732,7 +5732,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B135" s="19" t="str">
-        <x:v>Illumi</x:v>
+        <x:v>Kento Nanami</x:v>
       </x:c>
       <x:c r="C135" s="24" t="str">
         <x:f>D135&amp;"/"&amp;E135</x:f>
@@ -5751,27 +5751,27 @@
         <x:v>Magic</x:v>
       </x:c>
       <x:c r="H135" s="24" t="str">
-        <x:v>Evil</x:v>
+        <x:v>Good</x:v>
       </x:c>
       <x:c r="I135" s="18" t="str">
-        <x:v>Battlecry: Gain control of a minion with 2 HP or less</x:v>
+        <x:v>Battlecry: Set an enemy minion's HP to 1</x:v>
       </x:c>
       <x:c r="J135" s="18" t="str">
-        <x:v>Control</x:v>
+        <x:v>7:3 Ratio Technique</x:v>
       </x:c>
       <x:c r="K135" s="18" t="str">
-        <x:v>HxH</x:v>
+        <x:v>Jujutsu Kaisen</x:v>
       </x:c>
       <x:c r="L135" s="17" t="str">
-        <x:v>c131</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="136" ht="42" customHeight="1">
+        <x:v>c132</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="136" ht="60" customHeight="1">
       <x:c r="A136" s="21" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="B136" s="14" t="str">
-        <x:v>Kento Nanami</x:v>
+        <x:v>Knov</x:v>
       </x:c>
       <x:c r="C136" s="23" t="str">
         <x:f>D136&amp;"/"&amp;E136</x:f>
@@ -5784,7 +5784,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="F136" s="23" t="str">
-        <x:v>Epic</x:v>
+        <x:v>Mythic</x:v>
       </x:c>
       <x:c r="G136" s="23" t="str">
         <x:v>Magic</x:v>
@@ -5793,37 +5793,37 @@
         <x:v>Good</x:v>
       </x:c>
       <x:c r="I136" s="13" t="str">
-        <x:v>Battlecry: Set an enemy minion's HP to 1</x:v>
+        <x:v>Battlecry: Choose a friendly and an enemy minion to place in the pocket room, removing them from the board. After 2 turns, return the minion with the higher ATK</x:v>
       </x:c>
       <x:c r="J136" s="13" t="str">
-        <x:v>7:3 Ratio Technique</x:v>
+        <x:v>The Room</x:v>
       </x:c>
       <x:c r="K136" s="13" t="str">
-        <x:v>Jujutsu Kaisen</x:v>
+        <x:v>HxH</x:v>
       </x:c>
       <x:c r="L136" s="12" t="str">
-        <x:v>c132</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="137" ht="60" customHeight="1">
+        <x:v>c124</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="137" ht="44" customHeight="1">
       <x:c r="A137" s="22" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="B137" s="19" t="str">
-        <x:v>Knov</x:v>
+        <x:v>Knuckle</x:v>
       </x:c>
       <x:c r="C137" s="24" t="str">
         <x:f>D137&amp;"/"&amp;E137</x:f>
-        <x:v>1/1</x:v>
+        <x:v>0/3</x:v>
       </x:c>
       <x:c r="D137" s="22" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="E137" s="22" t="n">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F137" s="24" t="str">
-        <x:v>Mythic</x:v>
+        <x:v>Rare</x:v>
       </x:c>
       <x:c r="G137" s="24" t="str">
         <x:v>Magic</x:v>
@@ -5832,16 +5832,16 @@
         <x:v>Good</x:v>
       </x:c>
       <x:c r="I137" s="18" t="str">
-        <x:v>Battlecry: Choose a friendly and an enemy minion to place in the pocket room, removing them from the board. After 2 turns, return the minion with the higher ATK</x:v>
+        <x:v>Taunt. Passive: After the enemy minion attacks this minion, it can't attack for 2 turns</x:v>
       </x:c>
       <x:c r="J137" s="18" t="str">
-        <x:v>The Room</x:v>
+        <x:v>Taxes</x:v>
       </x:c>
       <x:c r="K137" s="18" t="str">
         <x:v>HxH</x:v>
       </x:c>
       <x:c r="L137" s="17" t="str">
-        <x:v>c124</x:v>
+        <x:v>c135</x:v>
       </x:c>
     </x:row>
     <x:row r="138" ht="44" customHeight="1">
@@ -5888,38 +5888,38 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B139" s="19" t="str">
-        <x:v>Margit the Fell Omen</x:v>
+        <x:v>Modern Tank</x:v>
       </x:c>
       <x:c r="C139" s="24" t="str">
         <x:f>D139&amp;"/"&amp;E139</x:f>
-        <x:v>1/1</x:v>
+        <x:v>2/2</x:v>
       </x:c>
       <x:c r="D139" s="22" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="E139" s="22" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F139" s="24" t="str">
         <x:v>Rare</x:v>
       </x:c>
       <x:c r="G139" s="24" t="str">
-        <x:v>Magic</x:v>
+        <x:v>Tech</x:v>
       </x:c>
       <x:c r="H139" s="24" t="str">
         <x:v>Neutral</x:v>
       </x:c>
       <x:c r="I139" s="18" t="str">
-        <x:v>Deathrattle: Summon Morgott, the Omen King (3/3)</x:v>
+        <x:v>Battlecry: Deal 1 damage to an enemy minion</x:v>
       </x:c>
       <x:c r="J139" s="18" t="str">
-        <x:v>The immovable</x:v>
+        <x:v>-</x:v>
       </x:c>
       <x:c r="K139" s="18" t="str">
-        <x:v>Elden Ring</x:v>
+        <x:v>Basic</x:v>
       </x:c>
       <x:c r="L139" s="17" t="str">
-        <x:v>c155</x:v>
+        <x:v>c139</x:v>
       </x:c>
     </x:row>
     <x:row r="140" ht="42" customHeight="1">
@@ -5927,38 +5927,38 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B140" s="14" t="str">
-        <x:v>Modern Tank</x:v>
+        <x:v>Morgott, the Omen King</x:v>
       </x:c>
       <x:c r="C140" s="23" t="str">
         <x:f>D140&amp;"/"&amp;E140</x:f>
-        <x:v>2/2</x:v>
+        <x:v>1/1</x:v>
       </x:c>
       <x:c r="D140" s="21" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E140" s="21" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F140" s="23" t="str">
         <x:v>Rare</x:v>
       </x:c>
       <x:c r="G140" s="23" t="str">
-        <x:v>Tech</x:v>
+        <x:v>Magic</x:v>
       </x:c>
       <x:c r="H140" s="23" t="str">
         <x:v>Neutral</x:v>
       </x:c>
       <x:c r="I140" s="13" t="str">
-        <x:v>Battlecry: Deal 1 damage to an enemy minion</x:v>
+        <x:v>Taunt. Battlecry: Summon Margit (1/1 with Taunt)</x:v>
       </x:c>
       <x:c r="J140" s="13" t="str">
-        <x:v>-</x:v>
+        <x:v>The immovable</x:v>
       </x:c>
       <x:c r="K140" s="13" t="str">
-        <x:v>Basic</x:v>
+        <x:v>Elden Ring</x:v>
       </x:c>
       <x:c r="L140" s="12" t="str">
-        <x:v>c139</x:v>
+        <x:v>c155</x:v>
       </x:c>
     </x:row>
     <x:row r="141" ht="42" customHeight="1">
@@ -6228,7 +6228,7 @@
         <x:v>Preparation beats power.</x:v>
       </x:c>
       <x:c r="K147" s="18" t="str">
-        <x:v>DCU</x:v>
+        <x:v>DCEU</x:v>
       </x:c>
       <x:c r="L147" s="17" t="str">
         <x:v>c005</x:v>
@@ -7658,7 +7658,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R926dd1d12fe64f49"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4a408c53735046e4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8378,7 +8378,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R03a016a13e3f48db"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re4d90fcead2b43f5"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>